<commit_message>
Implement festival data integration from Excel
</commit_message>
<xml_diff>
--- a/Таблица названий и имен.xlsx
+++ b/Таблица названий и имен.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\G\Info Cards Club\Диагностика Потенциала\Территория ИГРЫ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APK\id_diagnostic_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFA91477-219F-4C71-A68D-BAE39AC3464B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA48A9AC-0391-4704-B94B-49E1F4E23A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{92FBEEF1-FB5C-46C5-89DB-802F997D873A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>Олег Баранец</t>
   </si>
@@ -142,6 +142,15 @@
   </si>
   <si>
     <t>m00014</t>
+  </si>
+  <si>
+    <t>m00015</t>
+  </si>
+  <si>
+    <t>Наталия Баранец</t>
+  </si>
+  <si>
+    <t>Диагностика ИДП</t>
   </si>
 </sst>
 </file>
@@ -539,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C6917E-00A5-4ADF-B205-FF5BB8337890}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.28515625" customWidth="1"/>
@@ -560,10 +569,10 @@
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
@@ -699,6 +708,17 @@
       </c>
       <c r="C14" s="2" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update Festival Data (Excel import, age limit, UI updates)
</commit_message>
<xml_diff>
--- a/Таблица названий и имен.xlsx
+++ b/Таблица названий и имен.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APK\id_diagnostic_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA48A9AC-0391-4704-B94B-49E1F4E23A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF684BA-970A-4E73-AB54-58F869E35506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{92FBEEF1-FB5C-46C5-89DB-802F997D873A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>Олег Баранец</t>
   </si>
@@ -151,6 +151,21 @@
   </si>
   <si>
     <t>Диагностика ИДП</t>
+  </si>
+  <si>
+    <t>Имя</t>
+  </si>
+  <si>
+    <t>Игра</t>
+  </si>
+  <si>
+    <t>билет</t>
+  </si>
+  <si>
+    <t>количество игроков</t>
+  </si>
+  <si>
+    <t xml:space="preserve">возраст от </t>
   </si>
 </sst>
 </file>
@@ -548,177 +563,286 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C6917E-00A5-4ADF-B205-FF5BB8337890}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.140625" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="D2" s="2">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="D5" s="2">
         <v>10</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E5" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2">
+        <v>6</v>
+      </c>
+      <c r="E6" s="2">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2">
+        <v>6</v>
+      </c>
+      <c r="E7" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="D8" s="2">
+        <v>6</v>
+      </c>
+      <c r="E8" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="D9" s="2">
+        <v>6</v>
+      </c>
+      <c r="E9" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="D10" s="2">
+        <v>6</v>
+      </c>
+      <c r="E10" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="D11" s="2">
+        <v>5</v>
+      </c>
+      <c r="E11" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="D12" s="2">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="D13" s="2">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="D14" s="2">
+        <v>8</v>
+      </c>
+      <c r="E14" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="D15" s="2">
+        <v>5</v>
+      </c>
+      <c r="E15" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>39</v>
+      </c>
+      <c r="D16" s="2">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>